<commit_message>
Rebuild map with SFU building footprints
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/SFU_Burnaby_Study_Spots_Updated.xlsx
+++ b/SFU_Burnaby_Study_Spots_Updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kandi\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EAAFCAF-A615-4076-B6BE-76568A194A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73EEED62-FAE5-4D8B-889D-B2A980D8485F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Study Spots'!$A$1:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Study Spots'!$A$1:$H$14</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="74">
   <si>
     <t>Name</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Outlets</t>
   </si>
   <si>
-    <t>Notes / Verification</t>
-  </si>
-  <si>
     <t>Spot 1</t>
   </si>
   <si>
@@ -71,9 +68,6 @@
     <t>No</t>
   </si>
   <si>
-    <t>Size estimated at 20 sq ft/person; verify.</t>
-  </si>
-  <si>
     <t>Spot 2</t>
   </si>
   <si>
@@ -134,9 +128,6 @@
     <t>303</t>
   </si>
   <si>
-    <t>Size rounded from 70 × 20 sq ft/person; verify.</t>
-  </si>
-  <si>
     <t>Spot 9</t>
   </si>
   <si>
@@ -152,9 +143,6 @@
     <t>1500</t>
   </si>
   <si>
-    <t>Size estimated at 20 sq ft/person; verify. 'All day' retained as supplied.</t>
-  </si>
-  <si>
     <t>Spot 10</t>
   </si>
   <si>
@@ -167,42 +155,24 @@
     <t>3169</t>
   </si>
   <si>
-    <t>Hours retained as supplied; confirm whether AM/PM and days are correct. Size estimated.</t>
-  </si>
-  <si>
     <t>Spot 16</t>
   </si>
   <si>
     <t>ASB Public Lounge</t>
   </si>
   <si>
-    <t>ASB</t>
-  </si>
-  <si>
     <t>970.2</t>
   </si>
   <si>
     <t>970.3</t>
   </si>
   <si>
-    <t>Assumed same capacity as adjacent row based on supplied table; verify. Size estimated.</t>
-  </si>
-  <si>
     <t>Spot 23</t>
   </si>
   <si>
-    <t>Black Student Centre Lounge</t>
-  </si>
-  <si>
-    <t>MBC</t>
-  </si>
-  <si>
     <t>2270</t>
   </si>
   <si>
-    <t>Size estimated at 20 sq ft/person; verify. Hours/access should be confirmed.</t>
-  </si>
-  <si>
     <t>Item</t>
   </si>
   <si>
@@ -237,13 +207,52 @@
   </si>
   <si>
     <t>Confirm building hours, room access, and any special restrictions before displaying availability in SenseMap.</t>
+  </si>
+  <si>
+    <t>Latitudes/Longitudes</t>
+  </si>
+  <si>
+    <t>49.2787064,-122.9184207</t>
+  </si>
+  <si>
+    <t>49.2787064,-122.9184208</t>
+  </si>
+  <si>
+    <t>49.2787064,-122.9184209</t>
+  </si>
+  <si>
+    <t>49.2787064,-122.9184210</t>
+  </si>
+  <si>
+    <t>49.2787064,-122.9184211</t>
+  </si>
+  <si>
+    <t>49.2787064,-122.9184212</t>
+  </si>
+  <si>
+    <t>49.2787064,-122.9184213</t>
+  </si>
+  <si>
+    <t>49.2789103,-122.9174723</t>
+  </si>
+  <si>
+    <t>49.2774938,-122.9150385</t>
+  </si>
+  <si>
+    <t>MBC Black Student Centre Lounge</t>
+  </si>
+  <si>
+    <t>49.2787574,-122.9189221</t>
+  </si>
+  <si>
+    <t>49.279785842568984, -122.92228004067196</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -256,6 +265,12 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -271,7 +286,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -294,11 +309,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -308,6 +334,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -622,7 +651,6 @@
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="72" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.35">
@@ -650,25 +678,25 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
+      <c r="I1" s="4" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="F2" s="2">
         <v>150</v>
@@ -677,27 +705,27 @@
         <v>3000</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="F3" s="2">
         <v>50</v>
@@ -706,27 +734,27 @@
         <v>1000</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
+      </c>
+      <c r="I3" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="F4" s="2">
         <v>50</v>
@@ -735,27 +763,27 @@
         <v>1000</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="I4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F5" s="2">
         <v>24</v>
@@ -764,27 +792,27 @@
         <v>480</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="I5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F6" s="2">
         <v>10</v>
@@ -793,27 +821,27 @@
         <v>200</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="I6" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F7" s="2">
         <v>20</v>
@@ -822,27 +850,27 @@
         <v>400</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="I7" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="F8" s="2">
         <v>50</v>
@@ -851,27 +879,27 @@
         <v>1000</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="I8" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="F9" s="2">
         <v>70</v>
@@ -880,27 +908,27 @@
         <v>1400</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>36</v>
+        <v>20</v>
+      </c>
+      <c r="I9" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="F10" s="2">
         <v>50</v>
@@ -909,27 +937,27 @@
         <v>1000</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="F11" s="2">
         <v>70</v>
@@ -938,27 +966,27 @@
         <v>1400</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>47</v>
+        <v>20</v>
+      </c>
+      <c r="I11" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>50</v>
+        <v>44</v>
+      </c>
+      <c r="C12" s="2">
+        <v>9</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="F12" s="2">
         <v>15</v>
@@ -967,25 +995,25 @@
         <v>300</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+      <c r="I12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>50</v>
+        <v>44</v>
+      </c>
+      <c r="C13" s="2">
+        <v>9</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="F13" s="2">
         <v>15</v>
@@ -994,27 +1022,27 @@
         <v>300</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>53</v>
+        <v>20</v>
+      </c>
+      <c r="I13" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>56</v>
+        <v>71</v>
+      </c>
+      <c r="C14" s="2">
+        <v>9</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="F14" s="2">
         <v>68</v>
@@ -1023,15 +1051,17 @@
         <v>1360</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>58</v>
+        <v>20</v>
+      </c>
+      <c r="I14" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I14" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H14" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1046,50 +1076,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>